<commit_message>
refactor: streamline transaction processing and API interactions
This commit introduces a comprehensive refactoring of the end-to-end process. The core HTTP request workflows are standardized for improved error handling and consistency. All business logic components have been updated to align with the new interaction patterns, enhancing process robustness and maintainability.
</commit_message>
<xml_diff>
--- a/Data/Config.xlsx
+++ b/Data/Config.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="24931"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://uipath-my.sharepoint.com/personal/alexandra_veizu_uipath_com/Documents/Documents/Projects/REFrameworkNET5/StudioTemplates/REFramework/contentFiles/any/any/pt2/VisualBasic/Data/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\devcon\ACB.NewHireOnboarding.Performer\Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="1" documentId="13_ncr:1_{00D541BD-CB78-4D75-8532-9AD73E8C785E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{F8C54E24-BA5C-4BF9-8DAB-2778512EC11B}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3F1DF384-13BA-4D6D-A002-AB55A2417EB1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Settings" sheetId="1" r:id="rId1"/>
@@ -159,7 +159,7 @@
     <t xml:space="preserve">The maximum number of consecutive system exceptions was reached. </t>
   </si>
   <si>
-    <t>ProcessABCQueue</t>
+    <t>NewHireBenefitsPosting</t>
   </si>
 </sst>
 </file>
@@ -212,10 +212,10 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
   <cellXfs count="5">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -239,9 +239,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - 2022 Theme">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2013 - 2022">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -279,7 +279,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2013 - 2022">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -385,7 +385,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2013 - 2022">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -527,7 +527,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>

</xml_diff>